<commit_message>
added question and the visual aid
</commit_message>
<xml_diff>
--- a/docs/questions.xlsx
+++ b/docs/questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shrey\OneDrive\Desktop\SKULE_courses\Second_year\Sem 2\Probability and Statistics\MIE286---Group-033\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{892AC7AF-9AAA-4A91-94C3-9FCE0A474755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B87250-1943-4F95-8D35-EB6C008B6A25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="84">
   <si>
     <t>QuestionID</t>
   </si>
@@ -258,13 +258,29 @@
   </si>
   <si>
     <t>Q07 — Roses/flowers syllogism   → text,    Logic-Syllogism</t>
+  </si>
+  <si>
+    <t>family</t>
+  </si>
+  <si>
+    <t>Q08</t>
+  </si>
+  <si>
+    <t>A family has two children. You are told one of them is a boy. What is the probability both are boys? In percent, to nearest integer.</t>
+  </si>
+  <si>
+    <t>Conditional Probability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Possible combinations BB BG GB GG Given at least one boy, remove GG. Now the sample space becomes BB BG GB. Thus given the probability of 2 boys is Probability 1/3
+ </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -286,6 +302,17 @@
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -338,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -354,6 +381,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -657,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -708,7 +738,7 @@
       <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="6" t="s">
         <v>12</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -877,8 +907,36 @@
         <v>57</v>
       </c>
     </row>
+    <row r="9" spans="1:8" ht="50" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="2">
+        <v>33</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="G9" s="2">
+        <v>50</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>82</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
changed the timers and fixed index.html
</commit_message>
<xml_diff>
--- a/docs/questions.xlsx
+++ b/docs/questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shrey\OneDrive\Desktop\SKULE_courses\Second_year\Sem 2\Probability and Statistics\MIE286---Group-033\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1288DCBF-82D0-47FF-9B6C-EC2A53DA774F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D490A1-D060-42A0-9D74-37D6BC7ACAE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -291,17 +291,10 @@
     <t>C</t>
   </si>
   <si>
-    <t xml:space="preserve"> Average speed is total distance divided by total time, not the average of the two speeds.
-Let the distance one way be d.
-Time going = d / 60  
-Time returning = d / 30  
-Total distance = 2d  
-Total time = d/60 + d/30 = d/20  
-Average speed = Total distance / Total time  
-Average speed = 2d / (d/20) = 40 km/h thus the answer is B</t>
-  </si>
-  <si>
     <t>weeding out retards</t>
+  </si>
+  <si>
+    <t>Average speed is total distance divided by total time, not the average of the two speeds. Let the distance one way be d. Time going = d / 60 and Time returning = d / 30  and Total distance = 2d. Therefore, Total time = d/60 + d/30 = d/20. We know Average speed = Total distance / Total time. Thus, Average speed = 2d / (d/20) = 40 km/h thus the answer is B</t>
   </si>
 </sst>
 </file>
@@ -961,7 +954,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="162.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" ht="62.5" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>84</v>
       </c>
@@ -975,7 +968,7 @@
         <v>53</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>87</v>
@@ -984,7 +977,7 @@
         <v>88</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>